<commit_message>
Fix Excel template compatibility
</commit_message>
<xml_diff>
--- a/HV28_6T_WAT_12Point_VDD_Sweep_Template.xlsx
+++ b/HV28_6T_WAT_12Point_VDD_Sweep_Template.xlsx
@@ -90,7 +90,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -103,11 +103,20 @@
         <color rgb="00D2D2D7"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D2D2D7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -129,6 +138,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -203,60 +213,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PUManualWatTable" displayName="PUManualWatTable" ref="A1:I145" headerRowCount="1">
-  <autoFilter ref="A1:I145"/>
-  <tableColumns count="9">
-    <tableColumn id="1" name="Lot/Wafer"/>
-    <tableColumn id="2" name="Site"/>
-    <tableColumn id="3" name="Model VDD"/>
-    <tableColumn id="4" name="MOS"/>
-    <tableColumn id="5" name="Vt"/>
-    <tableColumn id="6" name="Vt Unit"/>
-    <tableColumn id="7" name="Idsat"/>
-    <tableColumn id="8" name="Idsat Unit"/>
-    <tableColumn id="9" name="Notes"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PGManualWatTable" displayName="PGManualWatTable" ref="A1:I145" headerRowCount="1">
-  <autoFilter ref="A1:I145"/>
-  <tableColumns count="9">
-    <tableColumn id="1" name="Lot/Wafer"/>
-    <tableColumn id="2" name="Site"/>
-    <tableColumn id="3" name="Model VDD"/>
-    <tableColumn id="4" name="MOS"/>
-    <tableColumn id="5" name="Vt"/>
-    <tableColumn id="6" name="Vt Unit"/>
-    <tableColumn id="7" name="Idsat"/>
-    <tableColumn id="8" name="Idsat Unit"/>
-    <tableColumn id="9" name="Notes"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PDManualWatTable" displayName="PDManualWatTable" ref="A1:I145" headerRowCount="1">
-  <autoFilter ref="A1:I145"/>
-  <tableColumns count="9">
-    <tableColumn id="1" name="Lot/Wafer"/>
-    <tableColumn id="2" name="Site"/>
-    <tableColumn id="3" name="Model VDD"/>
-    <tableColumn id="4" name="MOS"/>
-    <tableColumn id="5" name="Vt"/>
-    <tableColumn id="6" name="Vt Unit"/>
-    <tableColumn id="7" name="Idsat"/>
-    <tableColumn id="8" name="Idsat Unit"/>
-    <tableColumn id="9" name="Notes"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6516,9 +6472,6 @@
   </sheetData>
   <autoFilter ref="A1:I145"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -12496,9 +12449,6 @@
   </sheetData>
   <autoFilter ref="A1:I145"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -18476,9 +18426,6 @@
   </sheetData>
   <autoFilter ref="A1:I145"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -18518,10 +18465,10 @@
           <t>Lot/Wafer, Site, Model VDD, MOS, Vt, Vt Unit, Idsat, Idsat Unit and Notes.</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="8" t="n"/>
-      <c r="F4" s="8" t="n"/>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -18534,10 +18481,10 @@
           <t>PU contains PUL/PUR, PG contains PGL/PGR, and PD contains PDL/PDR.</t>
         </is>
       </c>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -18550,10 +18497,10 @@
           <t>S01-S12 are provided for every MOS and Model VDD, matching the manually organized table.</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -18566,10 +18513,10 @@
           <t>If S13-S17 become available, append them using the same columns; Python includes them automatically.</t>
         </is>
       </c>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -18582,10 +18529,10 @@
           <t>Data are grouped by Lot/Wafer + Model VDD + physical MOS.</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -18598,10 +18545,10 @@
           <t>The arithmetic mean of all valid rows is used as the Vt/Idsat input for each physical MOS.</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -18614,10 +18561,10 @@
           <t>N, median, sample standard deviation, minimum and maximum are retained in the output CSV.</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -18630,10 +18577,10 @@
           <t>Model VDD defaults to V. Vt accepts V/mV/uV/nV; Idsat accepts A/mA/uA/nA/pA.</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -18646,10 +18593,10 @@
           <t>Omit an unavailable row, or leave both Vt and Idsat blank. Do not fill only one value.</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="8" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -18662,10 +18609,10 @@
           <t>PU sample values follow the supplied manual table. PG/PD remain example data until replaced.</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>